<commit_message>
Add Nagasaki prefecture deep-dive (transport + tourism)
Enriched 長崎県 prefecture-wide plan and added 長崎市・佐世保市・
対馬市・平戸市 transport policies, plus tourism org detail for
長崎国際観光コンベンション協会 and 平戸観光協会.
</commit_message>
<xml_diff>
--- a/自治体施策DB/自治体交通観光施策DB.xlsx
+++ b/自治体施策DB/自治体交通観光施策DB.xlsx
@@ -16950,7 +16950,7 @@
       </c>
       <c r="G310" t="inlineStr">
         <is>
-          <t>観光地域づくり法人（地域DMO）として登録</t>
+          <t>「DMO NAGASAKI」として、観光資源の保護開発、内外観光客の誘致、コンベンション誘致支援、観光案内所運営等を実施。「長崎市サステナブルツーリズム～知識が景色を変えていく～」をテーマに高付加価値な滞在コンテンツを造成。飲食・宿泊事業者向けにビーガン・ハラル対応やデジタル発信のセミナー・伴走支援を実施し、クルーズ船客向け英語ガイド「Nagasaki Crew」を企画・運営。既存会員（約370社）に加え、長崎市観光まちづくりネットワーク（約370名）を新たに構築。</t>
         </is>
       </c>
       <c r="H310" t="inlineStr">
@@ -16965,7 +16965,12 @@
       </c>
       <c r="J310" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>深掘り調査（長崎県）</t>
         </is>
       </c>
     </row>
@@ -17049,12 +17054,12 @@
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>令和8年4月1日時点（現況）</t>
+          <t>地域DMO事業計画：令和6年3月</t>
         </is>
       </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t>観光地域づくり法人（地域DMO）として登録</t>
+          <t>自然・食・温泉・景観・文化的遺産（世界文化遺産）を活かしたテーマ観光の推進と観光DXに取組む。自ら車両を保有し、市内観光・長崎空港送迎の公共ライドシェア事業を実証運行。コンベンション開催事業費補助金の交付によりMICE誘致も支援。</t>
         </is>
       </c>
       <c r="H312" t="inlineStr">
@@ -17069,7 +17074,12 @@
       </c>
       <c r="J312" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>深掘り調査（長崎県）</t>
         </is>
       </c>
     </row>
@@ -18889,7 +18899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="2" min="1" max="1"/>
@@ -19911,37 +19921,37 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>地域公共交通計画（都道府県全域対象）</t>
+          <t>長崎県地域公共交通計画</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>令和8年3月末時点</t>
+          <t>令和8年3月改定（令和8年4月〜令和13年3月、5か年）※初版は令和5年3月策定</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>地域公共交通活性化再生法に基づき、長崎県が県内全市区町村を対象区域として地域公共交通計画を策定。人口減少・高齢化に対応した広域的な公共交通網の維持・再編を推進している。</t>
+          <t>3つの基本方針。(1)持続可能な幹線公共交通ネットワークの構築－バス路線(幹線)の役割整理、離島航路(31航路)・離島航空路(5航空路)の維持、地域鉄道(松浦鉄道・島原鉄道)及び西九州新幹線接続の長崎本線(江北〜諫早間)の維持、自動運転・AIオンデマンド交通など新技術活用、MaaSによる企画乗車券販売。(2)地域との共創による最適な地域モビリティの推進－フィーダー路線のデマンド化・モード転換、スクールバス等地域輸送資源の活用。(3)公共交通に関わる人材の確保・育成－運転士・整備士の確保、人材育成。数値目標(R12年度): 幹線バス年間輸送人員3,909,751人(現況4,073,893人)、コミュニティ交通導入21/21市町(現況19市町)、乗合バス運転士充足率96%(現況91%)。県内21市町中19市町が地域公共交通計画を策定済み(R7時点)。</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>国土交通省 地域公共交通計画の作成状況一覧（令和8年3月末時点）</t>
+          <t>長崎県地域公共交通計画 概要版（令和8年3月）</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>https://www.mlit.go.jp/sogoseisaku/transport/content/001965758.pdf</t>
+          <t>https://www.pref.nagasaki.jp/fs/9/7/8/6/_/________________.pdf</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>都道府県内の全市区町村を対象範囲に含む地域公共交通計画が策定されている（PDF一覧より抽出、令和8年3月末時点）。市区町村単位の個別策定状況は本PDFがベクトル文字の縦組みレイアウトで機械可読性が低いため、フェーズ1では未収集（今後個別に追加予定）。</t>
+          <t>深掘り調査（長崎県）。概要版PDF(7ページ)を精査済み。</t>
         </is>
       </c>
     </row>
@@ -20618,6 +20628,214 @@
       <c r="J33" s="2" t="inlineStr">
         <is>
           <t>深掘り調査（愛知県）。素案PDF(59ページ)のうち第1〜7章を精査。策定中のため今後内容が変わる可能性あり。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>長崎県</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>長崎市</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>交通</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>長崎市地域公共交通計画</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>令和8年3月策定（令和8年度〜12年度、5か年）※前計画は令和3年8月策定</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>国の「リ・デザイン」（地域公共交通の再構築）方針に対応し、利便性・持続可能性・生産性の高い地域公共交通への再構築を目指す。前計画に基づく「長崎市地域公共交通利便増進実施計画（東部地区）」（令和4年9月国認定）では、矢上バス停を拠点としたハブ&amp;スポーク型に路線再編し、乗継拠点整備や急行バス導入によりサービス改善。公共交通の徒歩圏カバー率は約77%で全国平均41%を大きく上回る。</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>長崎市地域公共交通計画を策定しました</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://www.city.nagasaki.lg.jp/page/5060.html</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>深掘り調査（長崎県）。全体像はページ記載分のみで、詳細な数値目標は本編PDF(18.16MB、未取得)に記載。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>長崎県</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>佐世保市、佐々町</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>交通</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>佐世保市・佐々町地域公共交通計画／利便増進実施計画</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>令和7年3月策定</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>隣接する佐々町と共同で地域公共交通計画・利便増進実施計画を策定。経由地を整理して分かりやすい路線に再編、日中時間帯の等間隔運行の導入、路線短縮、低床バスの導入、全国共通交通系ICカードの導入を実施。需要の低い地域はデマンド型タクシーへ転換。平成26年設置の「佐世保市地域公共交通活性化協議会」で協議・推進。</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>佐世保市・佐々町地域公共交通計画及び利便増進実施計画を策定</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://www.city.sasebo.lg.jp/tiikimirai/koukou/sasebosisazatyoutiikikoukyoukoutuukeikaku.html</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>深掘り調査（長崎県）。国認定は2件（No.30単独／No.97佐々町共同）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>長崎県</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>対馬市</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>交通</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>対馬市地域公共交通利便増進実施計画</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>令和7年6月策定（案）、実施期間令和7年度〜11年度（5か年）</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>幹線区間「厳原－対馬病院」の運行効率化によりバス路線事業全体の運行経費を年間約2,647万6千円削減。「対馬病院－仁位－比田勝港国際ターミナル」区間を増便（対馬病院－仁位：12便→14便、仁位－比田勝港国際ターミナル：10便→12便）し通学・通院・買い物の利便性を向上。対馬やまねこ空港・厳原港・比田勝港の国内外ターミナルとの乗継利便性を強化し、豊玉診療所・豊玉小学校・大浦への支線系統でラストワンマイルを確保。毎年度モニタリングを実施し改善施策を検討。</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>対馬市地域公共交通利便増進実施計画（案）</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://www.city.tsushima.nagasaki.jp/material/files/group/65/tusimasitiikikoukyoukoutuuribennzousinnzissikeikaku.pdf</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>深掘り調査（長崎県）。国交省認定リストNo.6の対象。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>長崎県</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>平戸市</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>交通</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>平戸市地域公共交通計画／利便増進実施計画</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>計画：令和7年3月策定</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>住民代表・交通事業者・行政の協議により、持続可能な公共交通の再構築の方向性を示すマスタープランとして策定。利便増進実施計画の第1弾事業として、生月バス「平戸高校線」の廃止に伴い、生月地区－中部地区間の路線再編を令和8年4月から実施予定。平戸観光協会による公共ライドシェア（市内観光・長崎空港送迎の実証運行）とも連携。</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>平戸市地域公共交通計画</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://www.city.hirado.nagasaki.jp/kurashi/life/sumai/koutu/2025-0425-0953-88.html</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>深掘り調査（長崎県）。国交省認定リストNo.40の対象。</t>
         </is>
       </c>
     </row>
@@ -63222,7 +63440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="2" min="1" max="1"/>
@@ -63452,6 +63670,28 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>長崎県への横展開: 長崎県地域公共交通計画を具体化、長崎市・佐世保市・対馬市・平戸市の交通施策を新規追加。観光は長崎国際観光コンベンション協会・平戸観光協会を深掘り</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>+1(更新)/+4(新規) 交通、+2(更新) 観光</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Claude（手動依頼対応）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add deep-dive priority ranking feature
New sheet ranks all 47 prefectures by a score combining certified
transport-project count (activity signal), municipality count
(market size), and plan-coverage rate (data feasibility). Already
deep-dived prefectures are kept at the bottom rather than removed.
</commit_message>
<xml_diff>
--- a/自治体施策DB/自治体交通観光施策DB.xlsx
+++ b/自治体施策DB/自治体交通観光施策DB.xlsx
@@ -11,16 +11,18 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交通施策" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交通_全国計画有無リサーチ" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交通_利便増進計画認定一覧" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="データソース一覧" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新履歴" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="深掘り優先度ランキング" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="データソース一覧" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新履歴" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'観光施策'!$A$1:$K$346</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'交通施策'!$A$1:$J$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'交通_全国計画有無リサーチ'!$A$1:$E$1715</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'交通_利便増進計画認定一覧'!$A$1:$F$119</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'データソース一覧'!$A$1:$F$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'更新履歴'!$A$1:$D$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'深掘り優先度ランキング'!$A$1:$H$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'データソース一覧'!$A$1:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'更新履歴'!$A$1:$D$2</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -91,7 +93,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -110,6 +112,12 @@
         <bgColor rgb="00305496"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -123,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -137,6 +145,7 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -502,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" style="2" min="1" max="1"/>
@@ -723,6 +732,44 @@
       <c r="A35" s="7" t="inlineStr">
         <is>
           <t>活動が活発な自治体を優先的に見つけたい場合の参考にしてください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>新シート「深掘り優先度ランキング」について:</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>次にどの都道府県を深掘りすべきかを、以下のスコアで機械的に算出したランキングです。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>スコア = 利便増進計画 認定件数×10 ＋ 市区町村数÷10 ＋ 地域公共交通計画カバー率(%)÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>認定件数（活発さ）を最も重視し、市区町村数（市場規模）とカバー率（情報の見つけやすさ）を補助指標としています。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>深掘り済みの都道府県は除外せず一覧の下部に残し、状況が変わればスコアを再計算して並び替えてください。</t>
         </is>
       </c>
     </row>
@@ -63133,6 +63180,1671 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>順位</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>都道府県</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>優先度スコア</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>利便増進計画 認定件数</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>市区町村数</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>地域公共交通計画カバー率</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>深掘り状況</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>スコアの根拠</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>北海道</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>81.2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" t="n">
+        <v>178</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>68.5%</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>認定6件×10 + 市区町村数178÷10 + カバー率69%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>新潟県</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>86.7%</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>認定6件×10 + 市区町村数30÷10 + カバー率87%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>長野県</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>74</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>認定5件×10 + 市区町村数74÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>高知県</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>認定5件×10 + 市区町村数34÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>広島県</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>23</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>認定5件×10 + 市区町村数23÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>福島県</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="D7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>58</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数58÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>宮崎県</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" t="n">
+        <v>26</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数26÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>大阪府</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="D9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>42</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>54.8%</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数42÷10 + カバー率55%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>大分県</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" t="n">
+        <v>18</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数18÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>岡山県</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" t="n">
+        <v>27</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>74.1%</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数27÷10 + カバー率74%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>石川県</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" t="n">
+        <v>19</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>84.2%</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数19÷10 + カバー率84%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>熊本県</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>45</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>認定3件×10 + 市区町村数45÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>千葉県</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" t="n">
+        <v>54</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>77.8%</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>認定3件×10 + 市区町村数54÷10 + カバー率78%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>奈良県</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="n">
+        <v>39</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>認定3件×10 + 市区町村数39÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>青森県</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" t="n">
+        <v>39</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>認定3件×10 + 市区町村数39÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>静岡県</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" t="n">
+        <v>35</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>認定3件×10 + 市区町村数35÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>佐賀県</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>37</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" t="n">
+        <v>20</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>認定3件×10 + 市区町村数20÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>鳥取県</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="n">
+        <v>19</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>63.2%</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>認定3件×10 + 市区町村数19÷10 + カバー率63%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>福岡県</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>31</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" t="n">
+        <v>60</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数60÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>埼玉県</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="n">
+        <v>62</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>69.4%</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数62÷10 + カバー率69%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>茨城県</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" t="n">
+        <v>44</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数44÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>岐阜県</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="D23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" t="n">
+        <v>42</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数42÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>宮城県</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="D24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" t="n">
+        <v>33</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数33÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>山形県</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" t="n">
+        <v>31</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数31÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>三重県</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="D26" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" t="n">
+        <v>29</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数29÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>兵庫県</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="D27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" t="n">
+        <v>41</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>75.6%</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数41÷10 + カバー率76%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>愛媛県</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>27</v>
+      </c>
+      <c r="D28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" t="n">
+        <v>20</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数20÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>香川県</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="D29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" t="n">
+        <v>17</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数17÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>山口県</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="D30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" t="n">
+        <v>19</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>94.7%</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数19÷10 + カバー率95%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>島根県</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>18</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>77.8%</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数18÷10 + カバー率78%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>福井県</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="D32" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" t="n">
+        <v>15</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>73.3%</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数15÷10 + カバー率73%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>鹿児島県</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>43</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数43÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>沖縄県</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>41</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数41÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>岩手県</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>33</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数33÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>群馬県</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>32</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数32÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>栃木県</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="n">
+        <v>25</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数25÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>徳島県</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="n">
+        <v>24</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数24÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>秋田県</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="n">
+        <v>24</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数24÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>滋賀県</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="n">
+        <v>18</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数18÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>富山県</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="n">
+        <v>14</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数14÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>京都府</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="n">
+        <v>26</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>69.2%</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数26÷10 + カバー率69%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>和歌山県</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>29</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>認定0件×10 + 市区町村数29÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>山梨県</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>26</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>認定0件×10 + 市区町村数26÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>神奈川県</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>33</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>63.6%</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>認定0件×10 + 市区町村数33÷10 + カバー率64%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>長崎県</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="D46" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E46" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G46" s="9" t="inlineStr">
+        <is>
+          <t>深掘り済み</t>
+        </is>
+      </c>
+      <c r="H46" s="9" t="inlineStr">
+        <is>
+          <t>認定6件×10 + 市区町村数21÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>愛知県</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="n">
+        <v>50.3</v>
+      </c>
+      <c r="D47" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E47" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>深掘り済み</t>
+        </is>
+      </c>
+      <c r="H47" s="9" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数53÷10 + カバー率100%÷20</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>東京都</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="D48" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E48" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>37.7%</t>
+        </is>
+      </c>
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>深掘り済み</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数61÷10 + カバー率38%÷20</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H48"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -63434,13 +65146,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="2" min="1" max="1"/>
@@ -63692,6 +65404,28 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>深掘り優先度を機械的に算出する「深掘り優先度ランキング」シートを新設（スコア=認定件数×10+市区町村数÷10+カバー率÷20）。次点は北海道（スコア81.2）</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>47都道府県</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Claude（優先順位付け機能の追加）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add feasibility score to the deep-dive priority ranking
New factor: 2pt for having a 政令指定都市 (designated city) plus
1pt per solo-certified transport project, on the theory that
larger/well-resourced municipalities publish plans in machine-
readable formats more reliably (validated against our own Aichi
deep-dive results, with the known 一宮市 counterexample noted).
</commit_message>
<xml_diff>
--- a/自治体施策DB/自治体交通観光施策DB.xlsx
+++ b/自治体施策DB/自治体交通観光施策DB.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'交通施策'!$A$1:$J$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'交通_全国計画有無リサーチ'!$A$1:$E$1715</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'交通_利便増進計画認定一覧'!$A$1:$F$119</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'深掘り優先度ランキング'!$A$1:$H$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'深掘り優先度ランキング'!$A$1:$K$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'データソース一覧'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'更新履歴'!$A$1:$D$2</definedName>
   </definedNames>
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:A48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" style="2" min="1" max="1"/>
@@ -770,6 +770,51 @@
       <c r="A41" s="7" t="inlineStr">
         <is>
           <t>深掘り済みの都道府県は除外せず一覧の下部に残し、状況が変わればスコアを再計算して並び替えてください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>「深掘り優先度ランキング」の改訂（実行可能性スコアの追加）:</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>スコア = 認定件数×10 ＋ 市区町村数÷10 ＋ カバー率(%)÷20 ＋ 実行可能性スコア×5</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>実行可能性スコア = (政令指定都市がある場合+2点) ＋ (認定案件のうち単独自治体の件数)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>「計画が存在するか」だけでなく「深掘りして具体的施策まで書ける可能性が高いか」を反映するために追加。</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>政令指定都市・中核市クラスの都市はPDFが通常レイアウトで機械可読な傾向が実績から確認できた一方、</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>一宮市（人口38万人の中核市）のように画像主体PDFで失敗した例もあり、あくまで確率を上げる代理指標である点に注意。</t>
         </is>
       </c>
     </row>
@@ -63180,17 +63225,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="56" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -63216,20 +63264,35 @@
       </c>
       <c r="E1" s="6" t="inlineStr">
         <is>
+          <t>うち単独自治体件数</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>政令指定都市</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
           <t>市区町村数</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>地域公共交通計画カバー率</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>実行可能性スコア</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>深掘り状況</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>スコアの根拠</t>
         </is>
@@ -63245,27 +63308,38 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>81.2</v>
+        <v>116.2</v>
       </c>
       <c r="D2" t="n">
         <v>6</v>
       </c>
       <c r="E2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
         <v>178</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>68.5%</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>認定6件×10 + 市区町村数178÷10 + カバー率69%÷20</t>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>認定6件×10 + 市区町村数178÷10 + カバー率69%÷20 + 実行可能性7点×5</t>
         </is>
       </c>
     </row>
@@ -63279,27 +63353,38 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>67.3</v>
+        <v>107.3</v>
       </c>
       <c r="D3" t="n">
         <v>6</v>
       </c>
       <c r="E3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
         <v>30</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>86.7%</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="n">
+        <v>8</v>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>認定6件×10 + 市区町村数30÷10 + カバー率87%÷20</t>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>認定6件×10 + 市区町村数30÷10 + カバー率87%÷20 + 実行可能性8点×5</t>
         </is>
       </c>
     </row>
@@ -63309,31 +63394,42 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>長野県</t>
+          <t>高知県</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>62.4</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="D4" t="n">
         <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>74</v>
+        <v>5</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>34</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>認定5件×10 + 市区町村数74÷10 + カバー率100%÷20</t>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>認定5件×10 + 市区町村数34÷10 + カバー率100%÷20 + 実行可能性5点×5</t>
         </is>
       </c>
     </row>
@@ -63343,31 +63439,42 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>高知県</t>
+          <t>広島県</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>58.4</v>
+        <v>82.3</v>
       </c>
       <c r="D5" t="n">
         <v>5</v>
       </c>
       <c r="E5" t="n">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>23</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="I5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>認定5件×10 + 市区町村数34÷10 + カバー率100%÷20</t>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>認定5件×10 + 市区町村数23÷10 + カバー率100%÷20 + 実行可能性5点×5</t>
         </is>
       </c>
     </row>
@@ -63377,31 +63484,42 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>広島県</t>
+          <t>大阪府</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>57.3</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>42</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>54.8%</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>6</v>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>認定5件×10 + 市区町村数23÷10 + カバー率100%÷20</t>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数42÷10 + カバー率55%÷20 + 実行可能性6点×5</t>
         </is>
       </c>
     </row>
@@ -63411,31 +63529,42 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>福島県</t>
+          <t>長野県</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>50.8</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E7" t="n">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>74</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="I7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>認定4件×10 + 市区町村数58÷10 + カバー率100%÷20</t>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>認定5件×10 + 市区町村数74÷10 + カバー率100%÷20 + 実行可能性2点×5</t>
         </is>
       </c>
     </row>
@@ -63445,31 +63574,42 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>宮崎県</t>
+          <t>岡山県</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>47.6</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="D8" t="n">
         <v>4</v>
       </c>
       <c r="E8" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>27</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>74.1%</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>認定4件×10 + 市区町村数26÷10 + カバー率100%÷20</t>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数27÷10 + カバー率74%÷20 + 実行可能性5点×5</t>
         </is>
       </c>
     </row>
@@ -63479,31 +63619,42 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>大阪府</t>
+          <t>千葉県</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>46.9</v>
+        <v>64.3</v>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>54.8%</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>54</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>77.8%</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>認定4件×10 + 市区町村数42÷10 + カバー率55%÷20</t>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>認定3件×10 + 市区町村数54÷10 + カバー率78%÷20 + 実行可能性5点×5</t>
         </is>
       </c>
     </row>
@@ -63513,31 +63664,42 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>大分県</t>
+          <t>静岡県</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>46.8</v>
+        <v>63.5</v>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>35</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="I10" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>認定4件×10 + 市区町村数18÷10 + カバー率100%÷20</t>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>認定3件×10 + 市区町村数35÷10 + カバー率100%÷20 + 実行可能性5点×5</t>
         </is>
       </c>
     </row>
@@ -63547,31 +63709,42 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>岡山県</t>
+          <t>石川県</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>46.4</v>
+        <v>61.1</v>
       </c>
       <c r="D11" t="n">
         <v>4</v>
       </c>
       <c r="E11" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>74.1%</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>19</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>84.2%</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J11" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>認定4件×10 + 市区町村数27÷10 + カバー率74%÷20</t>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数19÷10 + カバー率84%÷20 + 実行可能性3点×5</t>
         </is>
       </c>
     </row>
@@ -63581,31 +63754,42 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>石川県</t>
+          <t>熊本県</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>46.1</v>
+        <v>59.5</v>
       </c>
       <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>45</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>4</v>
       </c>
-      <c r="E12" t="n">
-        <v>19</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>84.2%</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>認定4件×10 + 市区町村数19÷10 + カバー率84%÷20</t>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>認定3件×10 + 市区町村数45÷10 + カバー率100%÷20 + 実行可能性4点×5</t>
         </is>
       </c>
     </row>
@@ -63615,31 +63799,42 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>熊本県</t>
+          <t>宮崎県</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>39.5</v>
+        <v>57.6</v>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>45</v>
+        <v>2</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>26</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="I13" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>認定3件×10 + 市区町村数45÷10 + カバー率100%÷20</t>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数26÷10 + カバー率100%÷20 + 実行可能性2点×5</t>
         </is>
       </c>
     </row>
@@ -63649,31 +63844,42 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>千葉県</t>
+          <t>福島県</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>39.3</v>
+        <v>55.8</v>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E14" t="n">
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>77.8%</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>58</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>認定3件×10 + 市区町村数54÷10 + カバー率78%÷20</t>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数58÷10 + カバー率100%÷20 + 実行可能性1点×5</t>
         </is>
       </c>
     </row>
@@ -63687,27 +63893,38 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>38.9</v>
+        <v>53.9</v>
       </c>
       <c r="D15" t="n">
         <v>3</v>
       </c>
       <c r="E15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
         <v>39</v>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="I15" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>認定3件×10 + 市区町村数39÷10 + カバー率100%÷20</t>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>認定3件×10 + 市区町村数39÷10 + カバー率100%÷20 + 実行可能性3点×5</t>
         </is>
       </c>
     </row>
@@ -63717,31 +63934,42 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>青森県</t>
+          <t>大分県</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>38.9</v>
+        <v>51.8</v>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E16" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>18</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>認定3件×10 + 市区町村数39÷10 + カバー率100%÷20</t>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数18÷10 + カバー率100%÷20 + 実行可能性1点×5</t>
         </is>
       </c>
     </row>
@@ -63751,31 +63979,42 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>静岡県</t>
+          <t>福岡県</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>38.5</v>
+        <v>51</v>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E17" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>60</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="I17" t="n">
+        <v>4</v>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>認定3件×10 + 市区町村数35÷10 + カバー率100%÷20</t>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数60÷10 + カバー率100%÷20 + 実行可能性4点×5</t>
         </is>
       </c>
     </row>
@@ -63785,31 +64024,42 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>佐賀県</t>
+          <t>埼玉県</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>37</v>
+        <v>49.7</v>
       </c>
       <c r="D18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E18" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>62</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>69.4%</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>4</v>
+      </c>
+      <c r="J18" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>認定3件×10 + 市区町村数20÷10 + カバー率100%÷20</t>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数62÷10 + カバー率69%÷20 + 実行可能性4点×5</t>
         </is>
       </c>
     </row>
@@ -63819,31 +64069,42 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>鳥取県</t>
+          <t>青森県</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>35.1</v>
+        <v>48.9</v>
       </c>
       <c r="D19" t="n">
         <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>63.2%</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>39</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>認定3件×10 + 市区町村数19÷10 + カバー率63%÷20</t>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>認定3件×10 + 市区町村数39÷10 + カバー率100%÷20 + 実行可能性2点×5</t>
         </is>
       </c>
     </row>
@@ -63853,31 +64114,42 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>福岡県</t>
+          <t>宮城県</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>31</v>
+        <v>48.3</v>
       </c>
       <c r="D20" t="n">
         <v>2</v>
       </c>
       <c r="E20" t="n">
-        <v>60</v>
+        <v>2</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>33</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="I20" t="n">
+        <v>4</v>
+      </c>
+      <c r="J20" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>認定2件×10 + 市区町村数60÷10 + カバー率100%÷20</t>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数33÷10 + カバー率100%÷20 + 実行可能性4点×5</t>
         </is>
       </c>
     </row>
@@ -63887,31 +64159,42 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>埼玉県</t>
+          <t>佐賀県</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>29.7</v>
+        <v>47</v>
       </c>
       <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="n">
         <v>2</v>
       </c>
-      <c r="E21" t="n">
-        <v>62</v>
-      </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>69.4%</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>20</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>2</v>
+      </c>
+      <c r="J21" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>認定2件×10 + 市区町村数62÷10 + カバー率69%÷20</t>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>認定3件×10 + 市区町村数20÷10 + カバー率100%÷20 + 実行可能性2点×5</t>
         </is>
       </c>
     </row>
@@ -63925,27 +64208,38 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>29.4</v>
+        <v>39.4</v>
       </c>
       <c r="D22" t="n">
         <v>2</v>
       </c>
       <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
         <v>44</v>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="I22" t="n">
+        <v>2</v>
+      </c>
+      <c r="J22" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>認定2件×10 + 市区町村数44÷10 + カバー率100%÷20</t>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数44÷10 + カバー率100%÷20 + 実行可能性2点×5</t>
         </is>
       </c>
     </row>
@@ -63955,31 +64249,42 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>岐阜県</t>
+          <t>山形県</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>29.2</v>
+        <v>38.1</v>
       </c>
       <c r="D23" t="n">
         <v>2</v>
       </c>
       <c r="E23" t="n">
-        <v>42</v>
+        <v>2</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>31</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="I23" t="n">
+        <v>2</v>
+      </c>
+      <c r="J23" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>認定2件×10 + 市区町村数42÷10 + カバー率100%÷20</t>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数31÷10 + カバー率100%÷20 + 実行可能性2点×5</t>
         </is>
       </c>
     </row>
@@ -63989,31 +64294,42 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>宮城県</t>
+          <t>兵庫県</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>28.3</v>
+        <v>37.9</v>
       </c>
       <c r="D24" t="n">
         <v>2</v>
       </c>
       <c r="E24" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>41</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>75.6%</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J24" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>認定2件×10 + 市区町村数33÷10 + カバー率100%÷20</t>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数41÷10 + カバー率76%÷20 + 実行可能性2点×5</t>
         </is>
       </c>
     </row>
@@ -64023,31 +64339,42 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>山形県</t>
+          <t>香川県</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>28.1</v>
+        <v>36.7</v>
       </c>
       <c r="D25" t="n">
         <v>2</v>
       </c>
       <c r="E25" t="n">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>17</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="I25" t="n">
+        <v>2</v>
+      </c>
+      <c r="J25" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>認定2件×10 + 市区町村数31÷10 + カバー率100%÷20</t>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数17÷10 + カバー率100%÷20 + 実行可能性2点×5</t>
         </is>
       </c>
     </row>
@@ -64057,31 +64384,42 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>三重県</t>
+          <t>山口県</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>27.9</v>
+        <v>36.6</v>
       </c>
       <c r="D26" t="n">
         <v>2</v>
       </c>
       <c r="E26" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>19</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>94.7%</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>2</v>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>認定2件×10 + 市区町村数29÷10 + カバー率100%÷20</t>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数19÷10 + カバー率95%÷20 + 実行可能性2点×5</t>
         </is>
       </c>
     </row>
@@ -64091,31 +64429,42 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>兵庫県</t>
+          <t>福井県</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>27.9</v>
+        <v>35.2</v>
       </c>
       <c r="D27" t="n">
         <v>2</v>
       </c>
       <c r="E27" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>75.6%</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>15</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>73.3%</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>認定2件×10 + 市区町村数41÷10 + カバー率76%÷20</t>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数15÷10 + カバー率73%÷20 + 実行可能性2点×5</t>
         </is>
       </c>
     </row>
@@ -64125,31 +64474,42 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>愛媛県</t>
+          <t>鳥取県</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>27</v>
+        <v>35.1</v>
       </c>
       <c r="D28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E28" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>19</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>63.2%</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>認定2件×10 + 市区町村数20÷10 + カバー率100%÷20</t>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>認定3件×10 + 市区町村数19÷10 + カバー率63%÷20 + 実行可能性0点×5</t>
         </is>
       </c>
     </row>
@@ -64159,31 +64519,42 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>香川県</t>
+          <t>岐阜県</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>26.7</v>
+        <v>34.2</v>
       </c>
       <c r="D29" t="n">
         <v>2</v>
       </c>
       <c r="E29" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>42</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="I29" t="n">
+        <v>1</v>
+      </c>
+      <c r="J29" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>認定2件×10 + 市区町村数17÷10 + カバー率100%÷20</t>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数42÷10 + カバー率100%÷20 + 実行可能性1点×5</t>
         </is>
       </c>
     </row>
@@ -64193,31 +64564,42 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>山口県</t>
+          <t>三重県</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>26.6</v>
+        <v>32.9</v>
       </c>
       <c r="D30" t="n">
         <v>2</v>
       </c>
       <c r="E30" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>94.7%</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>29</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J30" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>認定2件×10 + 市区町村数19÷10 + カバー率95%÷20</t>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数29÷10 + カバー率100%÷20 + 実行可能性1点×5</t>
         </is>
       </c>
     </row>
@@ -64227,31 +64609,42 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>島根県</t>
+          <t>京都府</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>25.7</v>
+        <v>31.1</v>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>77.8%</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>26</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>69.2%</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>3</v>
+      </c>
+      <c r="J31" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>認定2件×10 + 市区町村数18÷10 + カバー率78%÷20</t>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数26÷10 + カバー率69%÷20 + 実行可能性3点×5</t>
         </is>
       </c>
     </row>
@@ -64261,31 +64654,42 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>福井県</t>
+          <t>島根県</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25.2</v>
+        <v>30.7</v>
       </c>
       <c r="D32" t="n">
         <v>2</v>
       </c>
       <c r="E32" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>73.3%</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>18</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>77.8%</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J32" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>認定2件×10 + 市区町村数15÷10 + カバー率73%÷20</t>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数18÷10 + カバー率78%÷20 + 実行可能性1点×5</t>
         </is>
       </c>
     </row>
@@ -64295,31 +64699,42 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>鹿児島県</t>
+          <t>愛媛県</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>19.3</v>
+        <v>27</v>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E33" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>20</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="I33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>認定1件×10 + 市区町村数43÷10 + カバー率100%÷20</t>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>認定2件×10 + 市区町村数20÷10 + カバー率100%÷20 + 実行可能性0点×5</t>
         </is>
       </c>
     </row>
@@ -64329,31 +64744,42 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>沖縄県</t>
+          <t>鹿児島県</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>19.1</v>
+        <v>24.3</v>
       </c>
       <c r="D34" t="n">
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>43</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="I34" t="n">
+        <v>1</v>
+      </c>
+      <c r="J34" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>認定1件×10 + 市区町村数41÷10 + カバー率100%÷20</t>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数43÷10 + カバー率100%÷20 + 実行可能性1点×5</t>
         </is>
       </c>
     </row>
@@ -64363,31 +64789,42 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>岩手県</t>
+          <t>沖縄県</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>18.3</v>
+        <v>24.1</v>
       </c>
       <c r="D35" t="n">
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>41</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="I35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>認定1件×10 + 市区町村数33÷10 + カバー率100%÷20</t>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数41÷10 + カバー率100%÷20 + 実行可能性1点×5</t>
         </is>
       </c>
     </row>
@@ -64397,31 +64834,42 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>群馬県</t>
+          <t>岩手県</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>18.2</v>
+        <v>23.3</v>
       </c>
       <c r="D36" t="n">
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>33</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="I36" t="n">
+        <v>1</v>
+      </c>
+      <c r="J36" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>認定1件×10 + 市区町村数32÷10 + カバー率100%÷20</t>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数33÷10 + カバー率100%÷20 + 実行可能性1点×5</t>
         </is>
       </c>
     </row>
@@ -64431,31 +64879,42 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>栃木県</t>
+          <t>群馬県</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>17.5</v>
+        <v>23.2</v>
       </c>
       <c r="D37" t="n">
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>32</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="I37" t="n">
+        <v>1</v>
+      </c>
+      <c r="J37" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>認定1件×10 + 市区町村数25÷10 + カバー率100%÷20</t>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数32÷10 + カバー率100%÷20 + 実行可能性1点×5</t>
         </is>
       </c>
     </row>
@@ -64469,27 +64928,38 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>17.4</v>
+        <v>22.4</v>
       </c>
       <c r="D38" t="n">
         <v>1</v>
       </c>
       <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
         <v>24</v>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="I38" t="n">
+        <v>1</v>
+      </c>
+      <c r="J38" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>認定1件×10 + 市区町村数24÷10 + カバー率100%÷20</t>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数24÷10 + カバー率100%÷20 + 実行可能性1点×5</t>
         </is>
       </c>
     </row>
@@ -64503,27 +64973,38 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>17.4</v>
+        <v>22.4</v>
       </c>
       <c r="D39" t="n">
         <v>1</v>
       </c>
       <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
         <v>24</v>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="I39" t="n">
+        <v>1</v>
+      </c>
+      <c r="J39" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>認定1件×10 + 市区町村数24÷10 + カバー率100%÷20</t>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数24÷10 + カバー率100%÷20 + 実行可能性1点×5</t>
         </is>
       </c>
     </row>
@@ -64533,31 +65014,42 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>滋賀県</t>
+          <t>富山県</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>16.8</v>
+        <v>21.4</v>
       </c>
       <c r="D40" t="n">
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>14</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="I40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>認定1件×10 + 市区町村数18÷10 + カバー率100%÷20</t>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数14÷10 + カバー率100%÷20 + 実行可能性1点×5</t>
         </is>
       </c>
     </row>
@@ -64567,31 +65059,42 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>富山県</t>
+          <t>栃木県</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>16.4</v>
+        <v>17.5</v>
       </c>
       <c r="D41" t="n">
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>25</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>認定1件×10 + 市区町村数14÷10 + カバー率100%÷20</t>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数25÷10 + カバー率100%÷20 + 実行可能性0点×5</t>
         </is>
       </c>
     </row>
@@ -64601,31 +65104,42 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>京都府</t>
+          <t>滋賀県</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>16.1</v>
+        <v>16.8</v>
       </c>
       <c r="D42" t="n">
         <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>69.2%</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>18</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>認定1件×10 + 市区町村数26÷10 + カバー率69%÷20</t>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>認定1件×10 + 市区町村数18÷10 + カバー率100%÷20 + 実行可能性0点×5</t>
         </is>
       </c>
     </row>
@@ -64635,31 +65149,42 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>和歌山県</t>
+          <t>神奈川県</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>7.9</v>
+        <v>16.5</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>33</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>63.6%</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>2</v>
+      </c>
+      <c r="J43" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>認定0件×10 + 市区町村数29÷10 + カバー率100%÷20</t>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>認定0件×10 + 市区町村数33÷10 + カバー率64%÷20 + 実行可能性2点×5</t>
         </is>
       </c>
     </row>
@@ -64669,31 +65194,42 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>山梨県</t>
+          <t>和歌山県</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>7.6</v>
+        <v>7.9</v>
       </c>
       <c r="D44" t="n">
         <v>0</v>
       </c>
       <c r="E44" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>29</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>認定0件×10 + 市区町村数26÷10 + カバー率100%÷20</t>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>認定0件×10 + 市区町村数29÷10 + カバー率100%÷20 + 実行可能性0点×5</t>
         </is>
       </c>
     </row>
@@ -64703,31 +65239,42 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>神奈川県</t>
+          <t>山梨県</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>6.5</v>
+        <v>7.6</v>
       </c>
       <c r="D45" t="n">
         <v>0</v>
       </c>
       <c r="E45" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>63.6%</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>26</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>認定0件×10 + 市区町村数33÷10 + カバー率64%÷20</t>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>認定0件×10 + 市区町村数26÷10 + カバー率100%÷20 + 実行可能性0点×5</t>
         </is>
       </c>
     </row>
@@ -64741,27 +65288,38 @@
         </is>
       </c>
       <c r="C46" s="9" t="n">
-        <v>67.09999999999999</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="D46" s="9" t="n">
         <v>6</v>
       </c>
       <c r="E46" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G46" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="F46" s="9" t="inlineStr">
+      <c r="H46" s="9" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G46" s="9" t="inlineStr">
+      <c r="I46" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J46" s="9" t="inlineStr">
         <is>
           <t>深掘り済み</t>
         </is>
       </c>
-      <c r="H46" s="9" t="inlineStr">
-        <is>
-          <t>認定6件×10 + 市区町村数21÷10 + カバー率100%÷20</t>
+      <c r="K46" s="9" t="inlineStr">
+        <is>
+          <t>認定6件×10 + 市区町村数21÷10 + カバー率100%÷20 + 実行可能性5点×5</t>
         </is>
       </c>
     </row>
@@ -64775,27 +65333,38 @@
         </is>
       </c>
       <c r="C47" s="9" t="n">
-        <v>50.3</v>
+        <v>80.3</v>
       </c>
       <c r="D47" s="9" t="n">
         <v>4</v>
       </c>
       <c r="E47" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="G47" s="9" t="n">
         <v>53</v>
       </c>
-      <c r="F47" s="9" t="inlineStr">
+      <c r="H47" s="9" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G47" s="9" t="inlineStr">
+      <c r="I47" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J47" s="9" t="inlineStr">
         <is>
           <t>深掘り済み</t>
         </is>
       </c>
-      <c r="H47" s="9" t="inlineStr">
-        <is>
-          <t>認定4件×10 + 市区町村数53÷10 + カバー率100%÷20</t>
+      <c r="K47" s="9" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数53÷10 + カバー率100%÷20 + 実行可能性6点×5</t>
         </is>
       </c>
     </row>
@@ -64809,32 +65378,43 @@
         </is>
       </c>
       <c r="C48" s="9" t="n">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="D48" s="9" t="n">
         <v>4</v>
       </c>
       <c r="E48" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G48" s="9" t="n">
         <v>61</v>
       </c>
-      <c r="F48" s="9" t="inlineStr">
+      <c r="H48" s="9" t="inlineStr">
         <is>
           <t>37.7%</t>
         </is>
       </c>
-      <c r="G48" s="9" t="inlineStr">
+      <c r="I48" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="J48" s="9" t="inlineStr">
         <is>
           <t>深掘り済み</t>
         </is>
       </c>
-      <c r="H48" s="9" t="inlineStr">
-        <is>
-          <t>認定4件×10 + 市区町村数61÷10 + カバー率38%÷20</t>
+      <c r="K48" s="9" t="inlineStr">
+        <is>
+          <t>認定4件×10 + 市区町村数61÷10 + カバー率38%÷20 + 実行可能性4点×5</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H48"/>
+  <autoFilter ref="A1:K48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -65152,7 +65732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="2" min="1" max="1"/>
@@ -65426,6 +66006,28 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>深掘り優先度ランキングに「実行可能性スコア」（政令指定都市の有無＋単独認定件数）を追加し、計画の有無だけでなく深掘り成功率も反映。次点は北海道（スコア116.2）</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>47都道府県</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Claude（優先順位付けロジックの改善）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>